<commit_message>
feat: add project track field and require expert tags
- Add track field to projects (Индустриальный/Стартап/Образовательный/Научный)
- Validator normalizes different variants to 4 canonical Russian names
- Migration 026: add track column to projects table
- Update frontend: show track in ProjectsList
- Make expertise_tags required for experts (template + validation)
- Update test data generator to include tracks
- All tests pass (213 frontend)
</commit_message>
<xml_diff>
--- a/frontend/public/templates/projects_template.xlsx
+++ b/frontend/public/templates/projects_template.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -496,6 +496,11 @@
           <t>tags</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>track</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -523,6 +528,7 @@
           <t>NLP, Chatbot</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">

</xml_diff>